<commit_message>
Update 11 APR 2024
</commit_message>
<xml_diff>
--- a/CNTR_AT_2020.xlsx
+++ b/CNTR_AT_2020.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfcbs.warnier\Work Folders\Documents\Resilience dashboard project\ref-countries-2020-60m.geojson\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\jfcbs.warnier\Work Folders\Documents\Resilience dashboard project\ref-countries-2020-60m.geojson\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,6 +27,30 @@
     <author>JFCBS PLANS J9 CIMIC PPO WARNIER Axel OF-3</author>
   </authors>
   <commentList>
+    <comment ref="G14" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>JFCBS PLANS J9 CIMIC PPO WARNIER Axel OF-3:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+polygon closed but on the western border 1 line goes inwards</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G74" authorId="0" shapeId="0">
       <text>
         <r>
@@ -56,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="976">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="979">
   <si>
     <t>CNTR_ID</t>
   </si>
@@ -2971,9 +2995,6 @@
     <t>Y</t>
   </si>
   <si>
-    <t>Polygon_Ready</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
@@ -2984,6 +3005,18 @@
   </si>
   <si>
     <t>1051, 1043, 1031, 1009, 1312</t>
+  </si>
+  <si>
+    <t>999, 1000, 998, 1005, 1323</t>
+  </si>
+  <si>
+    <t>Rows to add</t>
+  </si>
+  <si>
+    <t>Rows to delete</t>
+  </si>
+  <si>
+    <t>64, 86, 113, 175, 391, 404, 433, 506</t>
   </si>
 </sst>
 </file>
@@ -3818,7 +3851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G241"/>
+  <dimension ref="A1:H241"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="50.7109375" bestFit="1" customWidth="1"/>
@@ -3826,9 +3859,10 @@
     <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.28515625" customWidth="1"/>
     <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3848,10 +3882,13 @@
         <v>969</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>971</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>976</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3868,7 +3905,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3885,7 +3922,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -3902,7 +3939,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -3919,7 +3956,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -3936,7 +3973,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -3956,10 +3993,10 @@
         <v>970</v>
       </c>
       <c r="G7" t="s">
-        <v>972</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -3976,7 +4013,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -3993,7 +4030,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>41</v>
       </c>
@@ -4010,7 +4047,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>45</v>
       </c>
@@ -4024,7 +4061,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>49</v>
       </c>
@@ -4041,7 +4078,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -4058,30 +4095,31 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="D14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="3" t="s">
         <v>970</v>
       </c>
-      <c r="G14" t="s">
-        <v>972</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G14" s="3" t="s">
+        <v>975</v>
+      </c>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -4098,7 +4136,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>66</v>
       </c>
@@ -4152,7 +4190,7 @@
         <v>970</v>
       </c>
       <c r="G18" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -4249,7 +4287,7 @@
         <v>970</v>
       </c>
       <c r="G23" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -4567,7 +4605,7 @@
         <v>970</v>
       </c>
       <c r="G41" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -4794,7 +4832,7 @@
         <v>970</v>
       </c>
       <c r="G54" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -4967,7 +5005,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>264</v>
       </c>
@@ -4984,7 +5022,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>268</v>
       </c>
@@ -5001,7 +5039,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>272</v>
       </c>
@@ -5021,10 +5059,10 @@
         <v>970</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>974</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>276</v>
       </c>
@@ -5041,7 +5079,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>280</v>
       </c>
@@ -5058,7 +5096,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>284</v>
       </c>
@@ -5075,7 +5113,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>288</v>
       </c>
@@ -5092,7 +5130,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>293</v>
       </c>
@@ -5109,7 +5147,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>297</v>
       </c>
@@ -5126,7 +5164,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>302</v>
       </c>
@@ -5142,12 +5180,17 @@
       <c r="E74" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="F74" s="3"/>
+      <c r="F74" s="3" t="s">
+        <v>970</v>
+      </c>
       <c r="G74" s="3" t="s">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+        <v>974</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>306</v>
       </c>
@@ -5164,7 +5207,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>312</v>
       </c>
@@ -5181,7 +5224,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>316</v>
       </c>
@@ -5198,7 +5241,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>320</v>
       </c>
@@ -5215,7 +5258,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>324</v>
       </c>
@@ -5232,7 +5275,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>329</v>
       </c>
@@ -5521,7 +5564,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>393</v>
       </c>
@@ -5538,7 +5581,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>397</v>
       </c>
@@ -5555,7 +5598,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>401</v>
       </c>
@@ -5572,7 +5615,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>405</v>
       </c>
@@ -5589,7 +5632,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>410</v>
       </c>
@@ -5606,7 +5649,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>414</v>
       </c>
@@ -5623,7 +5666,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>418</v>
       </c>
@@ -5640,7 +5683,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>422</v>
       </c>
@@ -5657,24 +5700,30 @@
         <v>425</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="C105" t="s">
+      <c r="C105" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="D105" t="s">
-        <v>9</v>
-      </c>
-      <c r="E105" t="s">
+      <c r="D105" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E105" s="2" t="s">
         <v>429</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F105" s="2" t="s">
+        <v>970</v>
+      </c>
+      <c r="G105" s="2">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>431</v>
       </c>
@@ -5691,7 +5740,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>435</v>
       </c>
@@ -5708,7 +5757,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>438</v>
       </c>
@@ -5725,7 +5774,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>442</v>
       </c>
@@ -5742,7 +5791,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>446</v>
       </c>
@@ -5759,7 +5808,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>450</v>
       </c>
@@ -5776,7 +5825,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>454</v>
       </c>

</xml_diff>